<commit_message>
updated fab outputs for light node
</commit_message>
<xml_diff>
--- a/RobotX2026/task-2/light-node/light-node.xlsx
+++ b/RobotX2026/task-2/light-node/light-node.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bd666c1b81e9ee1c/Documents/7-MIL/misc_hardware/RobotX2026/task-2/light-node/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="37" documentId="8_{74FAC293-BC0E-4791-84E4-3C3EAD8820A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8730BA84-F9E9-4521-85EC-322A1693F8D7}"/>
+  <xr:revisionPtr revIDLastSave="65" documentId="8_{74FAC293-BC0E-4791-84E4-3C3EAD8820A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ADE856A8-34D0-4634-B027-D87D3D294D23}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{8EDBA8C5-F057-4655-9CD6-696E9A273FD1}"/>
+    <workbookView xWindow="1536" yWindow="1536" windowWidth="17280" windowHeight="9960" xr2:uid="{8EDBA8C5-F057-4655-9CD6-696E9A273FD1}"/>
   </bookViews>
   <sheets>
     <sheet name="light-node" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="121">
   <si>
     <t>Line #</t>
   </si>
@@ -195,9 +195,6 @@
   </si>
   <si>
     <t>L1</t>
-  </si>
-  <si>
-    <t>Res</t>
   </si>
   <si>
     <t>SMD, RES0603</t>
@@ -365,6 +362,51 @@
   </si>
   <si>
     <t>GRM188R61E475KE11D</t>
+  </si>
+  <si>
+    <t>Res, 33</t>
+  </si>
+  <si>
+    <t>Res, 27</t>
+  </si>
+  <si>
+    <t>Res, 1k</t>
+  </si>
+  <si>
+    <t>Res, 10k</t>
+  </si>
+  <si>
+    <t>Res, 470</t>
+  </si>
+  <si>
+    <t>Res, 10</t>
+  </si>
+  <si>
+    <t>Res, 120</t>
+  </si>
+  <si>
+    <t>RC0603FR-0733RL</t>
+  </si>
+  <si>
+    <t>RC0603FR-0727RL</t>
+  </si>
+  <si>
+    <t>RC0603FR-071KL</t>
+  </si>
+  <si>
+    <t>RC0603FR-07470RL</t>
+  </si>
+  <si>
+    <t>RC0603FR-0710RL</t>
+  </si>
+  <si>
+    <t>RC0603FR-07120RL</t>
+  </si>
+  <si>
+    <t>YAGEO</t>
+  </si>
+  <si>
+    <t>SC1509-A4</t>
   </si>
 </sst>
 </file>
@@ -835,7 +877,7 @@
       </c>
       <c r="F2" s="1"/>
       <c r="G2" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
@@ -851,7 +893,7 @@
         <v>16</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>17</v>
@@ -863,7 +905,7 @@
         <v>18</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>20</v>
@@ -885,7 +927,7 @@
         <v>16</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>23</v>
@@ -919,7 +961,7 @@
         <v>16</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>24</v>
@@ -961,7 +1003,7 @@
       </c>
       <c r="F6" s="1"/>
       <c r="G6" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
@@ -999,7 +1041,7 @@
         <v>31</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>32</v>
@@ -1009,7 +1051,7 @@
       </c>
       <c r="F8" s="1"/>
       <c r="G8" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
@@ -1023,7 +1065,7 @@
         <v>33</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>34</v>
@@ -1033,7 +1075,7 @@
       </c>
       <c r="F9" s="1"/>
       <c r="G9" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
@@ -1141,7 +1183,7 @@
       </c>
       <c r="F13" s="1"/>
       <c r="G13" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
@@ -1152,22 +1194,22 @@
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="D14" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>53</v>
-      </c>
       <c r="E14" s="1">
         <v>1</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>54</v>
+        <v>119</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>55</v>
+        <v>113</v>
       </c>
       <c r="H14" s="2" t="s">
         <v>20</v>
@@ -1176,7 +1218,7 @@
         <v>43</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="K14" s="1">
         <v>0.1</v>
@@ -1190,22 +1232,22 @@
         <v>12</v>
       </c>
       <c r="B15" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="C15" s="2" t="s">
-        <v>52</v>
-      </c>
       <c r="D15" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E15" s="1">
         <v>2</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>54</v>
+        <v>119</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>55</v>
+        <v>114</v>
       </c>
       <c r="H15" s="2" t="s">
         <v>20</v>
@@ -1214,7 +1256,7 @@
         <v>43</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="K15" s="1">
         <v>0.1</v>
@@ -1228,22 +1270,22 @@
         <v>12</v>
       </c>
       <c r="B16" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>52</v>
-      </c>
       <c r="D16" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E16" s="1">
         <v>3</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>54</v>
+        <v>119</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>55</v>
+        <v>115</v>
       </c>
       <c r="H16" s="2" t="s">
         <v>20</v>
@@ -1252,7 +1294,7 @@
         <v>43</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="K16" s="1">
         <v>0.02</v>
@@ -1266,22 +1308,22 @@
         <v>12</v>
       </c>
       <c r="B17" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="C17" s="2" t="s">
-        <v>52</v>
-      </c>
       <c r="D17" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E17" s="1">
         <v>5</v>
       </c>
       <c r="F17" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G17" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>55</v>
       </c>
       <c r="H17" s="2" t="s">
         <v>20</v>
@@ -1290,7 +1332,7 @@
         <v>43</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="K17" s="1">
         <v>0.02</v>
@@ -1302,22 +1344,22 @@
     <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="C18" s="2" t="s">
-        <v>52</v>
-      </c>
       <c r="D18" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E18" s="1">
         <v>1</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>54</v>
+        <v>119</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>55</v>
+        <v>116</v>
       </c>
       <c r="H18" s="2" t="s">
         <v>20</v>
@@ -1326,7 +1368,7 @@
         <v>43</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="K18" s="1">
         <v>0.1</v>
@@ -1340,22 +1382,22 @@
         <v>12</v>
       </c>
       <c r="B19" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="C19" s="2" t="s">
-        <v>52</v>
-      </c>
       <c r="D19" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E19" s="1">
         <v>2</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>54</v>
+        <v>119</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>55</v>
+        <v>117</v>
       </c>
       <c r="H19" s="2" t="s">
         <v>20</v>
@@ -1364,7 +1406,7 @@
         <v>43</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="K19" s="1">
         <v>0.1</v>
@@ -1376,22 +1418,22 @@
     <row r="20" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
       <c r="B20" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="C20" s="2" t="s">
-        <v>52</v>
-      </c>
       <c r="D20" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E20" s="1">
         <v>1</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>54</v>
+        <v>119</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>55</v>
+        <v>118</v>
       </c>
       <c r="H20" s="2" t="s">
         <v>20</v>
@@ -1400,7 +1442,7 @@
         <v>43</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="K20" s="1">
         <v>0.1</v>
@@ -1412,20 +1454,20 @@
     <row r="21" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
       <c r="B21" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="D21" s="2" t="s">
         <v>64</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>65</v>
       </c>
       <c r="E21" s="1">
         <v>1</v>
       </c>
       <c r="F21" s="1"/>
       <c r="G21" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
@@ -1438,22 +1480,22 @@
         <v>12</v>
       </c>
       <c r="B22" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="D22" s="2" t="s">
         <v>67</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>68</v>
       </c>
       <c r="E22" s="1">
         <v>2</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H22" s="2" t="s">
         <v>20</v>
@@ -1462,7 +1504,7 @@
         <v>43</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="K22" s="1">
         <v>0.26</v>
@@ -1474,20 +1516,20 @@
     <row r="23" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
       <c r="B23" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="D23" s="2" t="s">
         <v>72</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>73</v>
       </c>
       <c r="E23" s="1">
         <v>1</v>
       </c>
       <c r="F23" s="1"/>
       <c r="G23" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
@@ -1498,19 +1540,21 @@
     <row r="24" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
       <c r="B24" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="D24" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="D24" s="2" t="s">
-        <v>76</v>
-      </c>
       <c r="E24" s="1">
         <v>1</v>
       </c>
       <c r="F24" s="1"/>
-      <c r="G24" s="1"/>
+      <c r="G24" s="1" t="s">
+        <v>120</v>
+      </c>
       <c r="H24" s="1"/>
       <c r="I24" s="1"/>
       <c r="J24" s="1"/>
@@ -1520,20 +1564,20 @@
     <row r="25" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
       <c r="B25" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="C25" s="2" t="s">
+      <c r="D25" s="2" t="s">
         <v>78</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>79</v>
       </c>
       <c r="E25" s="1">
         <v>1</v>
       </c>
       <c r="F25" s="1"/>
       <c r="G25" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H25" s="1"/>
       <c r="I25" s="1"/>
@@ -1544,20 +1588,20 @@
     <row r="26" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
       <c r="B26" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="D26" s="2" t="s">
         <v>81</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>82</v>
       </c>
       <c r="E26" s="1">
         <v>1</v>
       </c>
       <c r="F26" s="1"/>
       <c r="G26" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H26" s="1"/>
       <c r="I26" s="1"/>
@@ -1568,13 +1612,13 @@
     <row r="27" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
       <c r="B27" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C27" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="D27" s="2" t="s">
         <v>84</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>85</v>
       </c>
       <c r="E27" s="1">
         <v>1</v>
@@ -1590,20 +1634,20 @@
     <row r="28" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C28" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="C28" s="2" t="s">
+      <c r="D28" s="2" t="s">
         <v>87</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>88</v>
       </c>
       <c r="E28" s="1">
         <v>1</v>
       </c>
       <c r="F28" s="1"/>
       <c r="G28" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H28" s="1"/>
       <c r="I28" s="1"/>
@@ -1614,20 +1658,20 @@
     <row r="29" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C29" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="C29" s="2" t="s">
+      <c r="D29" s="2" t="s">
         <v>90</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>91</v>
       </c>
       <c r="E29" s="1">
         <v>1</v>
       </c>
       <c r="F29" s="1"/>
       <c r="G29" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H29" s="1"/>
       <c r="I29" s="1"/>
@@ -1638,20 +1682,20 @@
     <row r="30" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
       <c r="B30" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C30" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C30" s="2" t="s">
+      <c r="D30" s="2" t="s">
         <v>93</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>94</v>
       </c>
       <c r="E30" s="1">
         <v>1</v>
       </c>
       <c r="F30" s="1"/>
       <c r="G30" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H30" s="1"/>
       <c r="I30" s="1"/>

</xml_diff>